<commit_message>
Weekly data update 2026-06-02 (actuals + pace)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ferncrest_ok-fc_v2.xlsx
+++ b/ferncrest_ok-fc_v2.xlsx
@@ -4795,7 +4795,9 @@
       <c r="G6" s="179" t="n">
         <v>9427.34</v>
       </c>
-      <c r="H6" s="179" t="n"/>
+      <c r="H6" s="179" t="n">
+        <v>7805.25</v>
+      </c>
       <c r="I6" s="179" t="n"/>
       <c r="J6" s="179" t="n"/>
       <c r="K6" s="179" t="n"/>
@@ -5403,7 +5405,9 @@
       <c r="G24" s="179" t="n">
         <v>360</v>
       </c>
-      <c r="H24" s="179" t="n"/>
+      <c r="H24" s="179" t="n">
+        <v>372</v>
+      </c>
       <c r="I24" s="179" t="n"/>
       <c r="J24" s="179" t="n"/>
       <c r="K24" s="179" t="n"/>
@@ -5440,7 +5444,9 @@
       <c r="G25" s="179" t="n">
         <v>46</v>
       </c>
-      <c r="H25" s="179" t="n"/>
+      <c r="H25" s="179" t="n">
+        <v>27</v>
+      </c>
       <c r="I25" s="179" t="n"/>
       <c r="J25" s="179" t="n"/>
       <c r="K25" s="179" t="n"/>
@@ -5530,7 +5536,9 @@
       <c r="G27" s="179" t="n">
         <v>204.94</v>
       </c>
-      <c r="H27" s="179" t="n"/>
+      <c r="H27" s="179" t="n">
+        <v>289.08</v>
+      </c>
       <c r="I27" s="179" t="n"/>
       <c r="J27" s="179" t="n"/>
       <c r="K27" s="179" t="n"/>
@@ -5723,7 +5731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:N121"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="122" min="1" max="2"/>
@@ -7825,6 +7833,7 @@
         <v/>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="208" t="inlineStr">
         <is>
@@ -7833,30 +7842,30 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="122" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="122" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
       </c>
-      <c r="C53" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" t="n">
+      <c r="C53" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="122" t="n">
         <v>372</v>
       </c>
-      <c r="E53" t="n">
+      <c r="E53" s="122" t="n">
         <v>48</v>
       </c>
       <c r="F53" s="209">
         <f>IFERROR(E53/D53,0)</f>
         <v/>
       </c>
-      <c r="G53" t="n">
+      <c r="G53" s="122" t="n">
         <v>0</v>
       </c>
       <c r="H53" s="209">
@@ -7877,40 +7886,40 @@
       <c r="L53" s="210" t="n">
         <v>301.24</v>
       </c>
-      <c r="M53">
+      <c r="M53" s="122">
         <f>IFERROR(E53-VLOOKUP(B53,B$5:E52,4,0),"— first entry")</f>
         <v/>
       </c>
-      <c r="N53">
+      <c r="N53" s="122">
         <f>IF(E53=0,"— no bookings yet",IF(K53&lt;-0.05,"⚠️ Behind budget — review rate",IF(K53&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J53&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="122" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="122" t="inlineStr">
         <is>
           <t>Jun 2026</t>
         </is>
       </c>
-      <c r="C54" t="n">
+      <c r="C54" s="122" t="n">
         <v>4</v>
       </c>
-      <c r="D54" t="n">
+      <c r="D54" s="122" t="n">
         <v>360</v>
       </c>
-      <c r="E54" t="n">
+      <c r="E54" s="122" t="n">
         <v>49</v>
       </c>
       <c r="F54" s="209">
         <f>IFERROR(E54/D54,0)</f>
         <v/>
       </c>
-      <c r="G54" t="n">
+      <c r="G54" s="122" t="n">
         <v>0</v>
       </c>
       <c r="H54" s="209">
@@ -7931,40 +7940,40 @@
       <c r="L54" s="210" t="n">
         <v>254.48</v>
       </c>
-      <c r="M54">
+      <c r="M54" s="122">
         <f>IFERROR(E54-VLOOKUP(B54,B$5:E53,4,0),"— first entry")</f>
         <v/>
       </c>
-      <c r="N54">
+      <c r="N54" s="122">
         <f>IF(E54=0,"— no bookings yet",IF(K54&lt;-0.05,"⚠️ Behind budget — review rate",IF(K54&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J54&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="122" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="122" t="inlineStr">
         <is>
           <t>Jul 2026</t>
         </is>
       </c>
-      <c r="C55" t="n">
+      <c r="C55" s="122" t="n">
         <v>8</v>
       </c>
-      <c r="D55" t="n">
+      <c r="D55" s="122" t="n">
         <v>372</v>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="122" t="n">
         <v>10</v>
       </c>
       <c r="F55" s="209">
         <f>IFERROR(E55/D55,0)</f>
         <v/>
       </c>
-      <c r="G55" t="n">
+      <c r="G55" s="122" t="n">
         <v>0</v>
       </c>
       <c r="H55" s="209">
@@ -7985,40 +7994,40 @@
       <c r="L55" s="210" t="n">
         <v>395</v>
       </c>
-      <c r="M55">
+      <c r="M55" s="122">
         <f>IFERROR(E55-VLOOKUP(B55,B$5:E54,4,0),"— first entry")</f>
         <v/>
       </c>
-      <c r="N55">
+      <c r="N55" s="122">
         <f>IF(E55=0,"— no bookings yet",IF(K55&lt;-0.05,"⚠️ Behind budget — review rate",IF(K55&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J55&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="122" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="122" t="inlineStr">
         <is>
           <t>Aug 2026</t>
         </is>
       </c>
-      <c r="C56" t="n">
+      <c r="C56" s="122" t="n">
         <v>13</v>
       </c>
-      <c r="D56" t="n">
+      <c r="D56" s="122" t="n">
         <v>372</v>
       </c>
-      <c r="E56" t="n">
+      <c r="E56" s="122" t="n">
         <v>0</v>
       </c>
       <c r="F56" s="209">
         <f>IFERROR(E56/D56,0)</f>
         <v/>
       </c>
-      <c r="G56" t="n">
+      <c r="G56" s="122" t="n">
         <v>0</v>
       </c>
       <c r="H56" s="209">
@@ -8039,40 +8048,40 @@
       <c r="L56" s="210" t="n">
         <v>0</v>
       </c>
-      <c r="M56">
+      <c r="M56" s="122">
         <f>IFERROR(E56-VLOOKUP(B56,B$5:E55,4,0),"— first entry")</f>
         <v/>
       </c>
-      <c r="N56">
+      <c r="N56" s="122">
         <f>IF(E56=0,"— no bookings yet",IF(K56&lt;-0.05,"⚠️ Behind budget — review rate",IF(K56&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J56&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="122" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="122" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
       </c>
-      <c r="C57" t="n">
+      <c r="C57" s="122" t="n">
         <v>17</v>
       </c>
-      <c r="D57" t="n">
+      <c r="D57" s="122" t="n">
         <v>360</v>
       </c>
-      <c r="E57" t="n">
+      <c r="E57" s="122" t="n">
         <v>0</v>
       </c>
       <c r="F57" s="209">
         <f>IFERROR(E57/D57,0)</f>
         <v/>
       </c>
-      <c r="G57" t="n">
+      <c r="G57" s="122" t="n">
         <v>0</v>
       </c>
       <c r="H57" s="209">
@@ -8093,24 +8102,2687 @@
       <c r="L57" s="210" t="n">
         <v>0</v>
       </c>
-      <c r="M57">
+      <c r="M57" s="122">
         <f>IFERROR(E57-VLOOKUP(B57,B$5:E56,4,0),"— first entry")</f>
         <v/>
       </c>
-      <c r="N57">
+      <c r="N57" s="122">
         <f>IF(E57=0,"— no bookings yet",IF(K57&lt;-0.05,"⚠️ Behind budget — review rate",IF(K57&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J57&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
         <v/>
       </c>
     </row>
+    <row r="58"/>
+    <row r="59">
+      <c r="A59" s="208" t="inlineStr">
+        <is>
+          <t>▶  WEEK OF 2026-05-04  (script auto-populated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B60" s="122" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="C60" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E60" s="122" t="n">
+        <v>46</v>
+      </c>
+      <c r="F60" s="209">
+        <f>IFERROR(E60/D60,0)</f>
+        <v/>
+      </c>
+      <c r="G60" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="209">
+        <f>IFERROR(G60/D60,0)</f>
+        <v/>
+      </c>
+      <c r="I60" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J60" s="209">
+        <f>IFERROR(F60-H60,0)</f>
+        <v/>
+      </c>
+      <c r="K60" s="209">
+        <f>IFERROR(F60-I60,0)</f>
+        <v/>
+      </c>
+      <c r="L60" s="210" t="n">
+        <v>300.75</v>
+      </c>
+      <c r="M60" s="122">
+        <f>IFERROR(E60-VLOOKUP(B60,B$5:E59,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N60" s="122">
+        <f>IF(E60=0,"— no bookings yet",IF(K60&lt;-0.05,"⚠️ Behind budget — review rate",IF(K60&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J60&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B61" s="122" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="C61" s="122" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E61" s="122" t="n">
+        <v>49</v>
+      </c>
+      <c r="F61" s="209">
+        <f>IFERROR(E61/D61,0)</f>
+        <v/>
+      </c>
+      <c r="G61" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="209">
+        <f>IFERROR(G61/D61,0)</f>
+        <v/>
+      </c>
+      <c r="I61" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J61" s="209">
+        <f>IFERROR(F61-H61,0)</f>
+        <v/>
+      </c>
+      <c r="K61" s="209">
+        <f>IFERROR(F61-I61,0)</f>
+        <v/>
+      </c>
+      <c r="L61" s="210" t="n">
+        <v>254.48</v>
+      </c>
+      <c r="M61" s="122">
+        <f>IFERROR(E61-VLOOKUP(B61,B$5:E60,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N61" s="122">
+        <f>IF(E61=0,"— no bookings yet",IF(K61&lt;-0.05,"⚠️ Behind budget — review rate",IF(K61&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J61&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B62" s="122" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="C62" s="122" t="n">
+        <v>8</v>
+      </c>
+      <c r="D62" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E62" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="F62" s="209">
+        <f>IFERROR(E62/D62,0)</f>
+        <v/>
+      </c>
+      <c r="G62" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="209">
+        <f>IFERROR(G62/D62,0)</f>
+        <v/>
+      </c>
+      <c r="I62" s="209" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J62" s="209">
+        <f>IFERROR(F62-H62,0)</f>
+        <v/>
+      </c>
+      <c r="K62" s="209">
+        <f>IFERROR(F62-I62,0)</f>
+        <v/>
+      </c>
+      <c r="L62" s="210" t="n">
+        <v>392.33</v>
+      </c>
+      <c r="M62" s="122">
+        <f>IFERROR(E62-VLOOKUP(B62,B$5:E61,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N62" s="122">
+        <f>IF(E62=0,"— no bookings yet",IF(K62&lt;-0.05,"⚠️ Behind budget — review rate",IF(K62&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J62&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B63" s="122" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="C63" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="D63" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E63" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="209">
+        <f>IFERROR(E63/D63,0)</f>
+        <v/>
+      </c>
+      <c r="G63" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="209">
+        <f>IFERROR(G63/D63,0)</f>
+        <v/>
+      </c>
+      <c r="I63" s="209" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J63" s="209">
+        <f>IFERROR(F63-H63,0)</f>
+        <v/>
+      </c>
+      <c r="K63" s="209">
+        <f>IFERROR(F63-I63,0)</f>
+        <v/>
+      </c>
+      <c r="L63" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M63" s="122">
+        <f>IFERROR(E63-VLOOKUP(B63,B$5:E62,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N63" s="122">
+        <f>IF(E63=0,"— no bookings yet",IF(K63&lt;-0.05,"⚠️ Behind budget — review rate",IF(K63&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J63&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B64" s="122" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C64" s="122" t="n">
+        <v>17</v>
+      </c>
+      <c r="D64" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E64" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="209">
+        <f>IFERROR(E64/D64,0)</f>
+        <v/>
+      </c>
+      <c r="G64" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="209">
+        <f>IFERROR(G64/D64,0)</f>
+        <v/>
+      </c>
+      <c r="I64" s="209" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J64" s="209">
+        <f>IFERROR(F64-H64,0)</f>
+        <v/>
+      </c>
+      <c r="K64" s="209">
+        <f>IFERROR(F64-I64,0)</f>
+        <v/>
+      </c>
+      <c r="L64" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M64" s="122">
+        <f>IFERROR(E64-VLOOKUP(B64,B$5:E63,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N64" s="122">
+        <f>IF(E64=0,"— no bookings yet",IF(K64&lt;-0.05,"⚠️ Behind budget — review rate",IF(K64&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J64&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B65" s="122" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C65" s="122" t="n">
+        <v>21</v>
+      </c>
+      <c r="D65" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E65" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="209">
+        <f>IFERROR(E65/D65,0)</f>
+        <v/>
+      </c>
+      <c r="G65" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="209">
+        <f>IFERROR(G65/D65,0)</f>
+        <v/>
+      </c>
+      <c r="I65" s="209" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J65" s="209">
+        <f>IFERROR(F65-H65,0)</f>
+        <v/>
+      </c>
+      <c r="K65" s="209">
+        <f>IFERROR(F65-I65,0)</f>
+        <v/>
+      </c>
+      <c r="L65" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" s="122">
+        <f>IFERROR(E65-VLOOKUP(B65,B$5:E64,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N65" s="122">
+        <f>IF(E65=0,"— no bookings yet",IF(K65&lt;-0.05,"⚠️ Behind budget — review rate",IF(K65&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J65&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66"/>
+    <row r="67">
+      <c r="A67" s="208" t="inlineStr">
+        <is>
+          <t>▶  WEEK OF 2026-05-04  (script auto-populated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B68" s="122" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="C68" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E68" s="122" t="n">
+        <v>46</v>
+      </c>
+      <c r="F68" s="209">
+        <f>IFERROR(E68/D68,0)</f>
+        <v/>
+      </c>
+      <c r="G68" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="209">
+        <f>IFERROR(G68/D68,0)</f>
+        <v/>
+      </c>
+      <c r="I68" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J68" s="209">
+        <f>IFERROR(F68-H68,0)</f>
+        <v/>
+      </c>
+      <c r="K68" s="209">
+        <f>IFERROR(F68-I68,0)</f>
+        <v/>
+      </c>
+      <c r="L68" s="210" t="n">
+        <v>300.75</v>
+      </c>
+      <c r="M68" s="122">
+        <f>IFERROR(E68-VLOOKUP(B68,B$5:E67,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N68" s="122">
+        <f>IF(E68=0,"— no bookings yet",IF(K68&lt;-0.05,"⚠️ Behind budget — review rate",IF(K68&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J68&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B69" s="122" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="C69" s="122" t="n">
+        <v>4</v>
+      </c>
+      <c r="D69" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E69" s="122" t="n">
+        <v>49</v>
+      </c>
+      <c r="F69" s="209">
+        <f>IFERROR(E69/D69,0)</f>
+        <v/>
+      </c>
+      <c r="G69" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="209">
+        <f>IFERROR(G69/D69,0)</f>
+        <v/>
+      </c>
+      <c r="I69" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J69" s="209">
+        <f>IFERROR(F69-H69,0)</f>
+        <v/>
+      </c>
+      <c r="K69" s="209">
+        <f>IFERROR(F69-I69,0)</f>
+        <v/>
+      </c>
+      <c r="L69" s="210" t="n">
+        <v>254.48</v>
+      </c>
+      <c r="M69" s="122">
+        <f>IFERROR(E69-VLOOKUP(B69,B$5:E68,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N69" s="122">
+        <f>IF(E69=0,"— no bookings yet",IF(K69&lt;-0.05,"⚠️ Behind budget — review rate",IF(K69&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J69&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B70" s="122" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="C70" s="122" t="n">
+        <v>8</v>
+      </c>
+      <c r="D70" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E70" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="F70" s="209">
+        <f>IFERROR(E70/D70,0)</f>
+        <v/>
+      </c>
+      <c r="G70" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="209">
+        <f>IFERROR(G70/D70,0)</f>
+        <v/>
+      </c>
+      <c r="I70" s="209" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J70" s="209">
+        <f>IFERROR(F70-H70,0)</f>
+        <v/>
+      </c>
+      <c r="K70" s="209">
+        <f>IFERROR(F70-I70,0)</f>
+        <v/>
+      </c>
+      <c r="L70" s="210" t="n">
+        <v>392.33</v>
+      </c>
+      <c r="M70" s="122">
+        <f>IFERROR(E70-VLOOKUP(B70,B$5:E69,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N70" s="122">
+        <f>IF(E70=0,"— no bookings yet",IF(K70&lt;-0.05,"⚠️ Behind budget — review rate",IF(K70&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J70&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B71" s="122" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="C71" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="D71" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E71" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="209">
+        <f>IFERROR(E71/D71,0)</f>
+        <v/>
+      </c>
+      <c r="G71" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="209">
+        <f>IFERROR(G71/D71,0)</f>
+        <v/>
+      </c>
+      <c r="I71" s="209" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J71" s="209">
+        <f>IFERROR(F71-H71,0)</f>
+        <v/>
+      </c>
+      <c r="K71" s="209">
+        <f>IFERROR(F71-I71,0)</f>
+        <v/>
+      </c>
+      <c r="L71" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" s="122">
+        <f>IFERROR(E71-VLOOKUP(B71,B$5:E70,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N71" s="122">
+        <f>IF(E71=0,"— no bookings yet",IF(K71&lt;-0.05,"⚠️ Behind budget — review rate",IF(K71&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J71&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B72" s="122" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C72" s="122" t="n">
+        <v>17</v>
+      </c>
+      <c r="D72" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E72" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="209">
+        <f>IFERROR(E72/D72,0)</f>
+        <v/>
+      </c>
+      <c r="G72" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="209">
+        <f>IFERROR(G72/D72,0)</f>
+        <v/>
+      </c>
+      <c r="I72" s="209" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J72" s="209">
+        <f>IFERROR(F72-H72,0)</f>
+        <v/>
+      </c>
+      <c r="K72" s="209">
+        <f>IFERROR(F72-I72,0)</f>
+        <v/>
+      </c>
+      <c r="L72" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" s="122">
+        <f>IFERROR(E72-VLOOKUP(B72,B$5:E71,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N72" s="122">
+        <f>IF(E72=0,"— no bookings yet",IF(K72&lt;-0.05,"⚠️ Behind budget — review rate",IF(K72&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J72&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B73" s="122" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C73" s="122" t="n">
+        <v>21</v>
+      </c>
+      <c r="D73" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E73" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="209">
+        <f>IFERROR(E73/D73,0)</f>
+        <v/>
+      </c>
+      <c r="G73" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="209">
+        <f>IFERROR(G73/D73,0)</f>
+        <v/>
+      </c>
+      <c r="I73" s="209" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J73" s="209">
+        <f>IFERROR(F73-H73,0)</f>
+        <v/>
+      </c>
+      <c r="K73" s="209">
+        <f>IFERROR(F73-I73,0)</f>
+        <v/>
+      </c>
+      <c r="L73" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" s="122">
+        <f>IFERROR(E73-VLOOKUP(B73,B$5:E72,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N73" s="122">
+        <f>IF(E73=0,"— no bookings yet",IF(K73&lt;-0.05,"⚠️ Behind budget — review rate",IF(K73&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J73&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74"/>
+    <row r="75">
+      <c r="A75" s="208" t="inlineStr">
+        <is>
+          <t>▶  WEEK OF 2026-05-04  (script auto-populated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B76" s="122" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="C76" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E76" s="122" t="n">
+        <v>46</v>
+      </c>
+      <c r="F76" s="209">
+        <f>IFERROR(E76/D76,0)</f>
+        <v/>
+      </c>
+      <c r="G76" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="209">
+        <f>IFERROR(G76/D76,0)</f>
+        <v/>
+      </c>
+      <c r="I76" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J76" s="209">
+        <f>IFERROR(F76-H76,0)</f>
+        <v/>
+      </c>
+      <c r="K76" s="209">
+        <f>IFERROR(F76-I76,0)</f>
+        <v/>
+      </c>
+      <c r="L76" s="210" t="n">
+        <v>300.75</v>
+      </c>
+      <c r="M76" s="122">
+        <f>IFERROR(E76-VLOOKUP(B76,B$5:E75,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N76" s="122">
+        <f>IF(E76=0,"— no bookings yet",IF(K76&lt;-0.05,"⚠️ Behind budget — review rate",IF(K76&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J76&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B77" s="122" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="C77" s="122" t="n">
+        <v>4</v>
+      </c>
+      <c r="D77" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E77" s="122" t="n">
+        <v>49</v>
+      </c>
+      <c r="F77" s="209">
+        <f>IFERROR(E77/D77,0)</f>
+        <v/>
+      </c>
+      <c r="G77" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="209">
+        <f>IFERROR(G77/D77,0)</f>
+        <v/>
+      </c>
+      <c r="I77" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J77" s="209">
+        <f>IFERROR(F77-H77,0)</f>
+        <v/>
+      </c>
+      <c r="K77" s="209">
+        <f>IFERROR(F77-I77,0)</f>
+        <v/>
+      </c>
+      <c r="L77" s="210" t="n">
+        <v>254.48</v>
+      </c>
+      <c r="M77" s="122">
+        <f>IFERROR(E77-VLOOKUP(B77,B$5:E76,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N77" s="122">
+        <f>IF(E77=0,"— no bookings yet",IF(K77&lt;-0.05,"⚠️ Behind budget — review rate",IF(K77&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J77&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B78" s="122" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="C78" s="122" t="n">
+        <v>8</v>
+      </c>
+      <c r="D78" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E78" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="F78" s="209">
+        <f>IFERROR(E78/D78,0)</f>
+        <v/>
+      </c>
+      <c r="G78" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="209">
+        <f>IFERROR(G78/D78,0)</f>
+        <v/>
+      </c>
+      <c r="I78" s="209" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J78" s="209">
+        <f>IFERROR(F78-H78,0)</f>
+        <v/>
+      </c>
+      <c r="K78" s="209">
+        <f>IFERROR(F78-I78,0)</f>
+        <v/>
+      </c>
+      <c r="L78" s="210" t="n">
+        <v>392.33</v>
+      </c>
+      <c r="M78" s="122">
+        <f>IFERROR(E78-VLOOKUP(B78,B$5:E77,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N78" s="122">
+        <f>IF(E78=0,"— no bookings yet",IF(K78&lt;-0.05,"⚠️ Behind budget — review rate",IF(K78&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J78&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B79" s="122" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="C79" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="D79" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E79" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="209">
+        <f>IFERROR(E79/D79,0)</f>
+        <v/>
+      </c>
+      <c r="G79" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="209">
+        <f>IFERROR(G79/D79,0)</f>
+        <v/>
+      </c>
+      <c r="I79" s="209" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J79" s="209">
+        <f>IFERROR(F79-H79,0)</f>
+        <v/>
+      </c>
+      <c r="K79" s="209">
+        <f>IFERROR(F79-I79,0)</f>
+        <v/>
+      </c>
+      <c r="L79" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="122">
+        <f>IFERROR(E79-VLOOKUP(B79,B$5:E78,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N79" s="122">
+        <f>IF(E79=0,"— no bookings yet",IF(K79&lt;-0.05,"⚠️ Behind budget — review rate",IF(K79&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J79&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B80" s="122" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C80" s="122" t="n">
+        <v>17</v>
+      </c>
+      <c r="D80" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E80" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="209">
+        <f>IFERROR(E80/D80,0)</f>
+        <v/>
+      </c>
+      <c r="G80" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="209">
+        <f>IFERROR(G80/D80,0)</f>
+        <v/>
+      </c>
+      <c r="I80" s="209" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J80" s="209">
+        <f>IFERROR(F80-H80,0)</f>
+        <v/>
+      </c>
+      <c r="K80" s="209">
+        <f>IFERROR(F80-I80,0)</f>
+        <v/>
+      </c>
+      <c r="L80" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="122">
+        <f>IFERROR(E80-VLOOKUP(B80,B$5:E79,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N80" s="122">
+        <f>IF(E80=0,"— no bookings yet",IF(K80&lt;-0.05,"⚠️ Behind budget — review rate",IF(K80&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J80&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B81" s="122" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C81" s="122" t="n">
+        <v>21</v>
+      </c>
+      <c r="D81" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E81" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="209">
+        <f>IFERROR(E81/D81,0)</f>
+        <v/>
+      </c>
+      <c r="G81" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" s="209">
+        <f>IFERROR(G81/D81,0)</f>
+        <v/>
+      </c>
+      <c r="I81" s="209" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J81" s="209">
+        <f>IFERROR(F81-H81,0)</f>
+        <v/>
+      </c>
+      <c r="K81" s="209">
+        <f>IFERROR(F81-I81,0)</f>
+        <v/>
+      </c>
+      <c r="L81" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="122">
+        <f>IFERROR(E81-VLOOKUP(B81,B$5:E80,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N81" s="122">
+        <f>IF(E81=0,"— no bookings yet",IF(K81&lt;-0.05,"⚠️ Behind budget — review rate",IF(K81&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J81&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82"/>
+    <row r="83">
+      <c r="A83" s="208" t="inlineStr">
+        <is>
+          <t>▶  WEEK OF 2026-05-04  (script auto-populated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B84" s="122" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="C84" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E84" s="122" t="n">
+        <v>46</v>
+      </c>
+      <c r="F84" s="209">
+        <f>IFERROR(E84/D84,0)</f>
+        <v/>
+      </c>
+      <c r="G84" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="209">
+        <f>IFERROR(G84/D84,0)</f>
+        <v/>
+      </c>
+      <c r="I84" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J84" s="209">
+        <f>IFERROR(F84-H84,0)</f>
+        <v/>
+      </c>
+      <c r="K84" s="209">
+        <f>IFERROR(F84-I84,0)</f>
+        <v/>
+      </c>
+      <c r="L84" s="210" t="n">
+        <v>300.75</v>
+      </c>
+      <c r="M84" s="122">
+        <f>IFERROR(E84-VLOOKUP(B84,B$5:E83,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N84" s="122">
+        <f>IF(E84=0,"— no bookings yet",IF(K84&lt;-0.05,"⚠️ Behind budget — review rate",IF(K84&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J84&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B85" s="122" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="C85" s="122" t="n">
+        <v>4</v>
+      </c>
+      <c r="D85" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E85" s="122" t="n">
+        <v>49</v>
+      </c>
+      <c r="F85" s="209">
+        <f>IFERROR(E85/D85,0)</f>
+        <v/>
+      </c>
+      <c r="G85" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="209">
+        <f>IFERROR(G85/D85,0)</f>
+        <v/>
+      </c>
+      <c r="I85" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J85" s="209">
+        <f>IFERROR(F85-H85,0)</f>
+        <v/>
+      </c>
+      <c r="K85" s="209">
+        <f>IFERROR(F85-I85,0)</f>
+        <v/>
+      </c>
+      <c r="L85" s="210" t="n">
+        <v>254.48</v>
+      </c>
+      <c r="M85" s="122">
+        <f>IFERROR(E85-VLOOKUP(B85,B$5:E84,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N85" s="122">
+        <f>IF(E85=0,"— no bookings yet",IF(K85&lt;-0.05,"⚠️ Behind budget — review rate",IF(K85&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J85&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B86" s="122" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="C86" s="122" t="n">
+        <v>8</v>
+      </c>
+      <c r="D86" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E86" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="F86" s="209">
+        <f>IFERROR(E86/D86,0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="209">
+        <f>IFERROR(G86/D86,0)</f>
+        <v/>
+      </c>
+      <c r="I86" s="209" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J86" s="209">
+        <f>IFERROR(F86-H86,0)</f>
+        <v/>
+      </c>
+      <c r="K86" s="209">
+        <f>IFERROR(F86-I86,0)</f>
+        <v/>
+      </c>
+      <c r="L86" s="210" t="n">
+        <v>392.33</v>
+      </c>
+      <c r="M86" s="122">
+        <f>IFERROR(E86-VLOOKUP(B86,B$5:E85,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N86" s="122">
+        <f>IF(E86=0,"— no bookings yet",IF(K86&lt;-0.05,"⚠️ Behind budget — review rate",IF(K86&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J86&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B87" s="122" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="C87" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="D87" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E87" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="209">
+        <f>IFERROR(E87/D87,0)</f>
+        <v/>
+      </c>
+      <c r="G87" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="209">
+        <f>IFERROR(G87/D87,0)</f>
+        <v/>
+      </c>
+      <c r="I87" s="209" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J87" s="209">
+        <f>IFERROR(F87-H87,0)</f>
+        <v/>
+      </c>
+      <c r="K87" s="209">
+        <f>IFERROR(F87-I87,0)</f>
+        <v/>
+      </c>
+      <c r="L87" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" s="122">
+        <f>IFERROR(E87-VLOOKUP(B87,B$5:E86,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N87" s="122">
+        <f>IF(E87=0,"— no bookings yet",IF(K87&lt;-0.05,"⚠️ Behind budget — review rate",IF(K87&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J87&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B88" s="122" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C88" s="122" t="n">
+        <v>17</v>
+      </c>
+      <c r="D88" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E88" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="209">
+        <f>IFERROR(E88/D88,0)</f>
+        <v/>
+      </c>
+      <c r="G88" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="209">
+        <f>IFERROR(G88/D88,0)</f>
+        <v/>
+      </c>
+      <c r="I88" s="209" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J88" s="209">
+        <f>IFERROR(F88-H88,0)</f>
+        <v/>
+      </c>
+      <c r="K88" s="209">
+        <f>IFERROR(F88-I88,0)</f>
+        <v/>
+      </c>
+      <c r="L88" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" s="122">
+        <f>IFERROR(E88-VLOOKUP(B88,B$5:E87,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N88" s="122">
+        <f>IF(E88=0,"— no bookings yet",IF(K88&lt;-0.05,"⚠️ Behind budget — review rate",IF(K88&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J88&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B89" s="122" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C89" s="122" t="n">
+        <v>21</v>
+      </c>
+      <c r="D89" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E89" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="209">
+        <f>IFERROR(E89/D89,0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="209">
+        <f>IFERROR(G89/D89,0)</f>
+        <v/>
+      </c>
+      <c r="I89" s="209" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J89" s="209">
+        <f>IFERROR(F89-H89,0)</f>
+        <v/>
+      </c>
+      <c r="K89" s="209">
+        <f>IFERROR(F89-I89,0)</f>
+        <v/>
+      </c>
+      <c r="L89" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" s="122">
+        <f>IFERROR(E89-VLOOKUP(B89,B$5:E88,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N89" s="122">
+        <f>IF(E89=0,"— no bookings yet",IF(K89&lt;-0.05,"⚠️ Behind budget — review rate",IF(K89&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J89&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90"/>
+    <row r="91">
+      <c r="A91" s="208" t="inlineStr">
+        <is>
+          <t>▶  WEEK OF 2026-05-04  (script auto-populated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B92" s="122" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="C92" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E92" s="122" t="n">
+        <v>46</v>
+      </c>
+      <c r="F92" s="209">
+        <f>IFERROR(E92/D92,0)</f>
+        <v/>
+      </c>
+      <c r="G92" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" s="209">
+        <f>IFERROR(G92/D92,0)</f>
+        <v/>
+      </c>
+      <c r="I92" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J92" s="209">
+        <f>IFERROR(F92-H92,0)</f>
+        <v/>
+      </c>
+      <c r="K92" s="209">
+        <f>IFERROR(F92-I92,0)</f>
+        <v/>
+      </c>
+      <c r="L92" s="210" t="n">
+        <v>300.75</v>
+      </c>
+      <c r="M92" s="122">
+        <f>IFERROR(E92-VLOOKUP(B92,B$5:E91,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N92" s="122">
+        <f>IF(E92=0,"— no bookings yet",IF(K92&lt;-0.05,"⚠️ Behind budget — review rate",IF(K92&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J92&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B93" s="122" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="C93" s="122" t="n">
+        <v>4</v>
+      </c>
+      <c r="D93" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E93" s="122" t="n">
+        <v>49</v>
+      </c>
+      <c r="F93" s="209">
+        <f>IFERROR(E93/D93,0)</f>
+        <v/>
+      </c>
+      <c r="G93" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" s="209">
+        <f>IFERROR(G93/D93,0)</f>
+        <v/>
+      </c>
+      <c r="I93" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J93" s="209">
+        <f>IFERROR(F93-H93,0)</f>
+        <v/>
+      </c>
+      <c r="K93" s="209">
+        <f>IFERROR(F93-I93,0)</f>
+        <v/>
+      </c>
+      <c r="L93" s="210" t="n">
+        <v>254.48</v>
+      </c>
+      <c r="M93" s="122">
+        <f>IFERROR(E93-VLOOKUP(B93,B$5:E92,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N93" s="122">
+        <f>IF(E93=0,"— no bookings yet",IF(K93&lt;-0.05,"⚠️ Behind budget — review rate",IF(K93&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J93&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B94" s="122" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="C94" s="122" t="n">
+        <v>8</v>
+      </c>
+      <c r="D94" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E94" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="F94" s="209">
+        <f>IFERROR(E94/D94,0)</f>
+        <v/>
+      </c>
+      <c r="G94" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" s="209">
+        <f>IFERROR(G94/D94,0)</f>
+        <v/>
+      </c>
+      <c r="I94" s="209" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J94" s="209">
+        <f>IFERROR(F94-H94,0)</f>
+        <v/>
+      </c>
+      <c r="K94" s="209">
+        <f>IFERROR(F94-I94,0)</f>
+        <v/>
+      </c>
+      <c r="L94" s="210" t="n">
+        <v>392.33</v>
+      </c>
+      <c r="M94" s="122">
+        <f>IFERROR(E94-VLOOKUP(B94,B$5:E93,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N94" s="122">
+        <f>IF(E94=0,"— no bookings yet",IF(K94&lt;-0.05,"⚠️ Behind budget — review rate",IF(K94&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J94&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B95" s="122" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="C95" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="D95" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E95" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" s="209">
+        <f>IFERROR(E95/D95,0)</f>
+        <v/>
+      </c>
+      <c r="G95" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="209">
+        <f>IFERROR(G95/D95,0)</f>
+        <v/>
+      </c>
+      <c r="I95" s="209" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J95" s="209">
+        <f>IFERROR(F95-H95,0)</f>
+        <v/>
+      </c>
+      <c r="K95" s="209">
+        <f>IFERROR(F95-I95,0)</f>
+        <v/>
+      </c>
+      <c r="L95" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" s="122">
+        <f>IFERROR(E95-VLOOKUP(B95,B$5:E94,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N95" s="122">
+        <f>IF(E95=0,"— no bookings yet",IF(K95&lt;-0.05,"⚠️ Behind budget — review rate",IF(K95&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J95&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B96" s="122" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C96" s="122" t="n">
+        <v>17</v>
+      </c>
+      <c r="D96" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E96" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="209">
+        <f>IFERROR(E96/D96,0)</f>
+        <v/>
+      </c>
+      <c r="G96" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" s="209">
+        <f>IFERROR(G96/D96,0)</f>
+        <v/>
+      </c>
+      <c r="I96" s="209" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J96" s="209">
+        <f>IFERROR(F96-H96,0)</f>
+        <v/>
+      </c>
+      <c r="K96" s="209">
+        <f>IFERROR(F96-I96,0)</f>
+        <v/>
+      </c>
+      <c r="L96" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" s="122">
+        <f>IFERROR(E96-VLOOKUP(B96,B$5:E95,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N96" s="122">
+        <f>IF(E96=0,"— no bookings yet",IF(K96&lt;-0.05,"⚠️ Behind budget — review rate",IF(K96&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J96&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B97" s="122" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C97" s="122" t="n">
+        <v>21</v>
+      </c>
+      <c r="D97" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E97" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" s="209">
+        <f>IFERROR(E97/D97,0)</f>
+        <v/>
+      </c>
+      <c r="G97" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" s="209">
+        <f>IFERROR(G97/D97,0)</f>
+        <v/>
+      </c>
+      <c r="I97" s="209" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J97" s="209">
+        <f>IFERROR(F97-H97,0)</f>
+        <v/>
+      </c>
+      <c r="K97" s="209">
+        <f>IFERROR(F97-I97,0)</f>
+        <v/>
+      </c>
+      <c r="L97" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M97" s="122">
+        <f>IFERROR(E97-VLOOKUP(B97,B$5:E96,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N97" s="122">
+        <f>IF(E97=0,"— no bookings yet",IF(K97&lt;-0.05,"⚠️ Behind budget — review rate",IF(K97&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J97&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98"/>
+    <row r="99">
+      <c r="A99" s="208" t="inlineStr">
+        <is>
+          <t>▶  WEEK OF 2026-05-04  (script auto-populated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B100" s="122" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="C100" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E100" s="122" t="n">
+        <v>46</v>
+      </c>
+      <c r="F100" s="209">
+        <f>IFERROR(E100/D100,0)</f>
+        <v/>
+      </c>
+      <c r="G100" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="209">
+        <f>IFERROR(G100/D100,0)</f>
+        <v/>
+      </c>
+      <c r="I100" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J100" s="209">
+        <f>IFERROR(F100-H100,0)</f>
+        <v/>
+      </c>
+      <c r="K100" s="209">
+        <f>IFERROR(F100-I100,0)</f>
+        <v/>
+      </c>
+      <c r="L100" s="210" t="n">
+        <v>300.75</v>
+      </c>
+      <c r="M100" s="122">
+        <f>IFERROR(E100-VLOOKUP(B100,B$5:E99,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N100" s="122">
+        <f>IF(E100=0,"— no bookings yet",IF(K100&lt;-0.05,"⚠️ Behind budget — review rate",IF(K100&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J100&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B101" s="122" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="C101" s="122" t="n">
+        <v>4</v>
+      </c>
+      <c r="D101" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E101" s="122" t="n">
+        <v>49</v>
+      </c>
+      <c r="F101" s="209">
+        <f>IFERROR(E101/D101,0)</f>
+        <v/>
+      </c>
+      <c r="G101" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" s="209">
+        <f>IFERROR(G101/D101,0)</f>
+        <v/>
+      </c>
+      <c r="I101" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J101" s="209">
+        <f>IFERROR(F101-H101,0)</f>
+        <v/>
+      </c>
+      <c r="K101" s="209">
+        <f>IFERROR(F101-I101,0)</f>
+        <v/>
+      </c>
+      <c r="L101" s="210" t="n">
+        <v>254.48</v>
+      </c>
+      <c r="M101" s="122">
+        <f>IFERROR(E101-VLOOKUP(B101,B$5:E100,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N101" s="122">
+        <f>IF(E101=0,"— no bookings yet",IF(K101&lt;-0.05,"⚠️ Behind budget — review rate",IF(K101&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J101&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B102" s="122" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="C102" s="122" t="n">
+        <v>8</v>
+      </c>
+      <c r="D102" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E102" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="F102" s="209">
+        <f>IFERROR(E102/D102,0)</f>
+        <v/>
+      </c>
+      <c r="G102" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" s="209">
+        <f>IFERROR(G102/D102,0)</f>
+        <v/>
+      </c>
+      <c r="I102" s="209" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J102" s="209">
+        <f>IFERROR(F102-H102,0)</f>
+        <v/>
+      </c>
+      <c r="K102" s="209">
+        <f>IFERROR(F102-I102,0)</f>
+        <v/>
+      </c>
+      <c r="L102" s="210" t="n">
+        <v>392.33</v>
+      </c>
+      <c r="M102" s="122">
+        <f>IFERROR(E102-VLOOKUP(B102,B$5:E101,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N102" s="122">
+        <f>IF(E102=0,"— no bookings yet",IF(K102&lt;-0.05,"⚠️ Behind budget — review rate",IF(K102&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J102&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B103" s="122" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="C103" s="122" t="n">
+        <v>12</v>
+      </c>
+      <c r="D103" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E103" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" s="209">
+        <f>IFERROR(E103/D103,0)</f>
+        <v/>
+      </c>
+      <c r="G103" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" s="209">
+        <f>IFERROR(G103/D103,0)</f>
+        <v/>
+      </c>
+      <c r="I103" s="209" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J103" s="209">
+        <f>IFERROR(F103-H103,0)</f>
+        <v/>
+      </c>
+      <c r="K103" s="209">
+        <f>IFERROR(F103-I103,0)</f>
+        <v/>
+      </c>
+      <c r="L103" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M103" s="122">
+        <f>IFERROR(E103-VLOOKUP(B103,B$5:E102,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N103" s="122">
+        <f>IF(E103=0,"— no bookings yet",IF(K103&lt;-0.05,"⚠️ Behind budget — review rate",IF(K103&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J103&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B104" s="122" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C104" s="122" t="n">
+        <v>17</v>
+      </c>
+      <c r="D104" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E104" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F104" s="209">
+        <f>IFERROR(E104/D104,0)</f>
+        <v/>
+      </c>
+      <c r="G104" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" s="209">
+        <f>IFERROR(G104/D104,0)</f>
+        <v/>
+      </c>
+      <c r="I104" s="209" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J104" s="209">
+        <f>IFERROR(F104-H104,0)</f>
+        <v/>
+      </c>
+      <c r="K104" s="209">
+        <f>IFERROR(F104-I104,0)</f>
+        <v/>
+      </c>
+      <c r="L104" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M104" s="122">
+        <f>IFERROR(E104-VLOOKUP(B104,B$5:E103,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N104" s="122">
+        <f>IF(E104=0,"— no bookings yet",IF(K104&lt;-0.05,"⚠️ Behind budget — review rate",IF(K104&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J104&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B105" s="122" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C105" s="122" t="n">
+        <v>21</v>
+      </c>
+      <c r="D105" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E105" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" s="209">
+        <f>IFERROR(E105/D105,0)</f>
+        <v/>
+      </c>
+      <c r="G105" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" s="209">
+        <f>IFERROR(G105/D105,0)</f>
+        <v/>
+      </c>
+      <c r="I105" s="209" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J105" s="209">
+        <f>IFERROR(F105-H105,0)</f>
+        <v/>
+      </c>
+      <c r="K105" s="209">
+        <f>IFERROR(F105-I105,0)</f>
+        <v/>
+      </c>
+      <c r="L105" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M105" s="122">
+        <f>IFERROR(E105-VLOOKUP(B105,B$5:E104,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N105" s="122">
+        <f>IF(E105=0,"— no bookings yet",IF(K105&lt;-0.05,"⚠️ Behind budget — review rate",IF(K105&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J105&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106"/>
+    <row r="107">
+      <c r="A107" s="208" t="inlineStr">
+        <is>
+          <t>▶  WEEK OF 2026-05-17  (script auto-populated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B108" s="122" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="C108" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E108" s="122" t="n">
+        <v>45</v>
+      </c>
+      <c r="F108" s="209">
+        <f>IFERROR(E108/D108,0)</f>
+        <v/>
+      </c>
+      <c r="G108" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" s="209">
+        <f>IFERROR(G108/D108,0)</f>
+        <v/>
+      </c>
+      <c r="I108" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J108" s="209">
+        <f>IFERROR(F108-H108,0)</f>
+        <v/>
+      </c>
+      <c r="K108" s="209">
+        <f>IFERROR(F108-I108,0)</f>
+        <v/>
+      </c>
+      <c r="L108" s="210" t="n">
+        <v>274.86</v>
+      </c>
+      <c r="M108" s="122">
+        <f>IFERROR(E108-VLOOKUP(B108,B$5:E107,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N108" s="122">
+        <f>IF(E108=0,"— no bookings yet",IF(K108&lt;-0.05,"⚠️ Behind budget — review rate",IF(K108&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J108&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B109" s="122" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="C109" s="122" t="n">
+        <v>2</v>
+      </c>
+      <c r="D109" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E109" s="122" t="n">
+        <v>56</v>
+      </c>
+      <c r="F109" s="209">
+        <f>IFERROR(E109/D109,0)</f>
+        <v/>
+      </c>
+      <c r="G109" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" s="209">
+        <f>IFERROR(G109/D109,0)</f>
+        <v/>
+      </c>
+      <c r="I109" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J109" s="209">
+        <f>IFERROR(F109-H109,0)</f>
+        <v/>
+      </c>
+      <c r="K109" s="209">
+        <f>IFERROR(F109-I109,0)</f>
+        <v/>
+      </c>
+      <c r="L109" s="210" t="n">
+        <v>260.33</v>
+      </c>
+      <c r="M109" s="122">
+        <f>IFERROR(E109-VLOOKUP(B109,B$5:E108,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N109" s="122">
+        <f>IF(E109=0,"— no bookings yet",IF(K109&lt;-0.05,"⚠️ Behind budget — review rate",IF(K109&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J109&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B110" s="122" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="C110" s="122" t="n">
+        <v>6</v>
+      </c>
+      <c r="D110" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E110" s="122" t="n">
+        <v>19</v>
+      </c>
+      <c r="F110" s="209">
+        <f>IFERROR(E110/D110,0)</f>
+        <v/>
+      </c>
+      <c r="G110" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" s="209">
+        <f>IFERROR(G110/D110,0)</f>
+        <v/>
+      </c>
+      <c r="I110" s="209" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J110" s="209">
+        <f>IFERROR(F110-H110,0)</f>
+        <v/>
+      </c>
+      <c r="K110" s="209">
+        <f>IFERROR(F110-I110,0)</f>
+        <v/>
+      </c>
+      <c r="L110" s="210" t="n">
+        <v>395.32</v>
+      </c>
+      <c r="M110" s="122">
+        <f>IFERROR(E110-VLOOKUP(B110,B$5:E109,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N110" s="122">
+        <f>IF(E110=0,"— no bookings yet",IF(K110&lt;-0.05,"⚠️ Behind budget — review rate",IF(K110&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J110&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B111" s="122" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="C111" s="122" t="n">
+        <v>10</v>
+      </c>
+      <c r="D111" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E111" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" s="209">
+        <f>IFERROR(E111/D111,0)</f>
+        <v/>
+      </c>
+      <c r="G111" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" s="209">
+        <f>IFERROR(G111/D111,0)</f>
+        <v/>
+      </c>
+      <c r="I111" s="209" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J111" s="209">
+        <f>IFERROR(F111-H111,0)</f>
+        <v/>
+      </c>
+      <c r="K111" s="209">
+        <f>IFERROR(F111-I111,0)</f>
+        <v/>
+      </c>
+      <c r="L111" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" s="122">
+        <f>IFERROR(E111-VLOOKUP(B111,B$5:E110,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N111" s="122">
+        <f>IF(E111=0,"— no bookings yet",IF(K111&lt;-0.05,"⚠️ Behind budget — review rate",IF(K111&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J111&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B112" s="122" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C112" s="122" t="n">
+        <v>15</v>
+      </c>
+      <c r="D112" s="122" t="n">
+        <v>360</v>
+      </c>
+      <c r="E112" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" s="209">
+        <f>IFERROR(E112/D112,0)</f>
+        <v/>
+      </c>
+      <c r="G112" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" s="209">
+        <f>IFERROR(G112/D112,0)</f>
+        <v/>
+      </c>
+      <c r="I112" s="209" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J112" s="209">
+        <f>IFERROR(F112-H112,0)</f>
+        <v/>
+      </c>
+      <c r="K112" s="209">
+        <f>IFERROR(F112-I112,0)</f>
+        <v/>
+      </c>
+      <c r="L112" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" s="122">
+        <f>IFERROR(E112-VLOOKUP(B112,B$5:E111,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N112" s="122">
+        <f>IF(E112=0,"— no bookings yet",IF(K112&lt;-0.05,"⚠️ Behind budget — review rate",IF(K112&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J112&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="122" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B113" s="122" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C113" s="122" t="n">
+        <v>19</v>
+      </c>
+      <c r="D113" s="122" t="n">
+        <v>372</v>
+      </c>
+      <c r="E113" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" s="209">
+        <f>IFERROR(E113/D113,0)</f>
+        <v/>
+      </c>
+      <c r="G113" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" s="209">
+        <f>IFERROR(G113/D113,0)</f>
+        <v/>
+      </c>
+      <c r="I113" s="209" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J113" s="209">
+        <f>IFERROR(F113-H113,0)</f>
+        <v/>
+      </c>
+      <c r="K113" s="209">
+        <f>IFERROR(F113-I113,0)</f>
+        <v/>
+      </c>
+      <c r="L113" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" s="122">
+        <f>IFERROR(E113-VLOOKUP(B113,B$5:E112,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N113" s="122">
+        <f>IF(E113=0,"— no bookings yet",IF(K113&lt;-0.05,"⚠️ Behind budget — review rate",IF(K113&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J113&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="208" t="inlineStr">
+        <is>
+          <t>▶  WEEK OF 2026-05-17  (script auto-populated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" t="n">
+        <v>372</v>
+      </c>
+      <c r="E116" t="n">
+        <v>55</v>
+      </c>
+      <c r="F116" s="209">
+        <f>IFERROR(E116/D116,0)</f>
+        <v/>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" s="209">
+        <f>IFERROR(G116/D116,0)</f>
+        <v/>
+      </c>
+      <c r="I116" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J116" s="209">
+        <f>IFERROR(F116-H116,0)</f>
+        <v/>
+      </c>
+      <c r="K116" s="209">
+        <f>IFERROR(F116-I116,0)</f>
+        <v/>
+      </c>
+      <c r="L116" s="210" t="n">
+        <v>265.45</v>
+      </c>
+      <c r="M116">
+        <f>IFERROR(E116-VLOOKUP(B116,B$5:E115,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N116">
+        <f>IF(E116=0,"— no bookings yet",IF(K116&lt;-0.05,"⚠️ Behind budget — review rate",IF(K116&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J116&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>2</v>
+      </c>
+      <c r="D117" t="n">
+        <v>360</v>
+      </c>
+      <c r="E117" t="n">
+        <v>69</v>
+      </c>
+      <c r="F117" s="209">
+        <f>IFERROR(E117/D117,0)</f>
+        <v/>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" s="209">
+        <f>IFERROR(G117/D117,0)</f>
+        <v/>
+      </c>
+      <c r="I117" s="209" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J117" s="209">
+        <f>IFERROR(F117-H117,0)</f>
+        <v/>
+      </c>
+      <c r="K117" s="209">
+        <f>IFERROR(F117-I117,0)</f>
+        <v/>
+      </c>
+      <c r="L117" s="210" t="n">
+        <v>256.09</v>
+      </c>
+      <c r="M117">
+        <f>IFERROR(E117-VLOOKUP(B117,B$5:E116,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N117">
+        <f>IF(E117=0,"— no bookings yet",IF(K117&lt;-0.05,"⚠️ Behind budget — review rate",IF(K117&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J117&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>6</v>
+      </c>
+      <c r="D118" t="n">
+        <v>372</v>
+      </c>
+      <c r="E118" t="n">
+        <v>22</v>
+      </c>
+      <c r="F118" s="209">
+        <f>IFERROR(E118/D118,0)</f>
+        <v/>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" s="209">
+        <f>IFERROR(G118/D118,0)</f>
+        <v/>
+      </c>
+      <c r="I118" s="209" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J118" s="209">
+        <f>IFERROR(F118-H118,0)</f>
+        <v/>
+      </c>
+      <c r="K118" s="209">
+        <f>IFERROR(F118-I118,0)</f>
+        <v/>
+      </c>
+      <c r="L118" s="210" t="n">
+        <v>398.09</v>
+      </c>
+      <c r="M118">
+        <f>IFERROR(E118-VLOOKUP(B118,B$5:E117,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N118">
+        <f>IF(E118=0,"— no bookings yet",IF(K118&lt;-0.05,"⚠️ Behind budget — review rate",IF(K118&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J118&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>10</v>
+      </c>
+      <c r="D119" t="n">
+        <v>372</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0</v>
+      </c>
+      <c r="F119" s="209">
+        <f>IFERROR(E119/D119,0)</f>
+        <v/>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" s="209">
+        <f>IFERROR(G119/D119,0)</f>
+        <v/>
+      </c>
+      <c r="I119" s="209" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J119" s="209">
+        <f>IFERROR(F119-H119,0)</f>
+        <v/>
+      </c>
+      <c r="K119" s="209">
+        <f>IFERROR(F119-I119,0)</f>
+        <v/>
+      </c>
+      <c r="L119" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M119">
+        <f>IFERROR(E119-VLOOKUP(B119,B$5:E118,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N119">
+        <f>IF(E119=0,"— no bookings yet",IF(K119&lt;-0.05,"⚠️ Behind budget — review rate",IF(K119&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J119&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>15</v>
+      </c>
+      <c r="D120" t="n">
+        <v>360</v>
+      </c>
+      <c r="E120" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" s="209">
+        <f>IFERROR(E120/D120,0)</f>
+        <v/>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" s="209">
+        <f>IFERROR(G120/D120,0)</f>
+        <v/>
+      </c>
+      <c r="I120" s="209" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J120" s="209">
+        <f>IFERROR(F120-H120,0)</f>
+        <v/>
+      </c>
+      <c r="K120" s="209">
+        <f>IFERROR(F120-I120,0)</f>
+        <v/>
+      </c>
+      <c r="L120" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120">
+        <f>IFERROR(E120-VLOOKUP(B120,B$5:E119,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N120">
+        <f>IF(E120=0,"— no bookings yet",IF(K120&lt;-0.05,"⚠️ Behind budget — review rate",IF(K120&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J120&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>19</v>
+      </c>
+      <c r="D121" t="n">
+        <v>372</v>
+      </c>
+      <c r="E121" t="n">
+        <v>0</v>
+      </c>
+      <c r="F121" s="209">
+        <f>IFERROR(E121/D121,0)</f>
+        <v/>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" s="209">
+        <f>IFERROR(G121/D121,0)</f>
+        <v/>
+      </c>
+      <c r="I121" s="209" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J121" s="209">
+        <f>IFERROR(F121-H121,0)</f>
+        <v/>
+      </c>
+      <c r="K121" s="209">
+        <f>IFERROR(F121-I121,0)</f>
+        <v/>
+      </c>
+      <c r="L121" s="210" t="n">
+        <v>0</v>
+      </c>
+      <c r="M121">
+        <f>IFERROR(E121-VLOOKUP(B121,B$5:E120,4,0),"— first entry")</f>
+        <v/>
+      </c>
+      <c r="N121">
+        <f>IF(E121=0,"— no bookings yet",IF(K121&lt;-0.05,"⚠️ Behind budget — review rate",IF(K121&gt;0.05,"✅ Ahead — hold rate or push ADR",IF(J121&lt;-0.03,"↓ Soft vs LY — monitor","◼ On track"))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="17">
+    <mergeCell ref="A67:N67"/>
     <mergeCell ref="A31:N31"/>
+    <mergeCell ref="A91:N91"/>
+    <mergeCell ref="A83:N83"/>
     <mergeCell ref="A4:N4"/>
     <mergeCell ref="A38:N38"/>
     <mergeCell ref="A24:N24"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A52:N52"/>
+    <mergeCell ref="A59:N59"/>
+    <mergeCell ref="A115:N115"/>
+    <mergeCell ref="A107:N107"/>
+    <mergeCell ref="A99:N99"/>
     <mergeCell ref="A45:N45"/>
+    <mergeCell ref="A75:N75"/>
     <mergeCell ref="A14:N14"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -9400,7 +12072,7 @@
         </is>
       </c>
       <c r="B11" s="140" t="n">
-        <v>57632.67</v>
+        <v>65437.92</v>
       </c>
       <c r="C11" s="165" t="inlineStr">
         <is>
@@ -9540,7 +12212,7 @@
         </is>
       </c>
       <c r="B18" s="238" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="C18" s="165" t="inlineStr">
         <is>
@@ -9580,7 +12252,7 @@
         </is>
       </c>
       <c r="B20" s="238" t="n">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="C20" s="165" t="inlineStr">
         <is>
@@ -9620,7 +12292,7 @@
         </is>
       </c>
       <c r="B22" s="238" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C22" s="165" t="inlineStr">
         <is>
@@ -9660,7 +12332,7 @@
         </is>
       </c>
       <c r="B24" s="122" t="n">
-        <v>250</v>
+        <v>277</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="123">
@@ -9670,7 +12342,7 @@
         </is>
       </c>
       <c r="B25" s="122" t="n">
-        <v>0.1736</v>
+        <v>0.1529</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="123">
@@ -9680,7 +12352,7 @@
         </is>
       </c>
       <c r="B26" s="122" t="n">
-        <v>230.53</v>
+        <v>236.24</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="123">
@@ -9690,7 +12362,7 @@
         </is>
       </c>
       <c r="B27" s="122" t="n">
-        <v>40.02</v>
+        <v>36.11</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="123">
@@ -9700,7 +12372,7 @@
         </is>
       </c>
       <c r="B28" s="122" t="n">
-        <v>0.129</v>
+        <v>0.1478</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="123">
@@ -9710,7 +12382,7 @@
         </is>
       </c>
       <c r="B29" s="122" t="n">
-        <v>301.24</v>
+        <v>265.45</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="123">
@@ -9720,7 +12392,7 @@
         </is>
       </c>
       <c r="B30" s="122" t="n">
-        <v>0.1361</v>
+        <v>0.1917</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="123">
@@ -9730,7 +12402,7 @@
         </is>
       </c>
       <c r="B31" s="122" t="n">
-        <v>254.48</v>
+        <v>256.09</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="123">
@@ -9740,7 +12412,7 @@
         </is>
       </c>
       <c r="B32" s="122" t="n">
-        <v>0.0269</v>
+        <v>0.0591</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="123">
@@ -9750,7 +12422,7 @@
         </is>
       </c>
       <c r="B33" s="122" t="n">
-        <v>395</v>
+        <v>398.09</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="123">
@@ -9761,7 +12433,7 @@
       </c>
       <c r="B34" s="122" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>

</xml_diff>